<commit_message>
Atualização de base (+ CNH) — 03/10/2026 21:23
</commit_message>
<xml_diff>
--- a/dados/metas.xlsx
+++ b/dados/metas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro.sa\Documents\dashboard-oportunidades\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DED88F9D-4825-4696-B598-D9528DCAD3AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E00F2B0-5AFF-45AD-9623-FC58A57C3230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONSULTOR" sheetId="1" r:id="rId1"/>
@@ -14690,7 +14690,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R254" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
@@ -22232,26 +22231,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f76aa77c-8923-4724-9a6d-d588cc513697">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="89c54d5b-05ac-45d5-9242-aabb385cc5ad" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B96036E30F13644F923D207E371C305D" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1d197ceb99055fd1a93a3a14aec1bdd8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f76aa77c-8923-4724-9a6d-d588cc513697" xmlns:ns3="89c54d5b-05ac-45d5-9242-aabb385cc5ad" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5b86266bfd619f312673123d0bd20d23" ns2:_="" ns3:_="">
     <xsd:import namespace="f76aa77c-8923-4724-9a6d-d588cc513697"/>
@@ -22446,32 +22425,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F919D1BA-3E11-4877-AEE4-5A5340B7B50A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="89c54d5b-05ac-45d5-9242-aabb385cc5ad"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="f76aa77c-8923-4724-9a6d-d588cc513697"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5CFE981-CBAC-4360-B0CE-AB3235A33930}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f76aa77c-8923-4724-9a6d-d588cc513697">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="89c54d5b-05ac-45d5-9242-aabb385cc5ad" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8BDC8EFC-C946-4B3C-B84E-1270F018751C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -22488,4 +22462,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5CFE981-CBAC-4360-B0CE-AB3235A33930}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F919D1BA-3E11-4877-AEE4-5A5340B7B50A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="89c54d5b-05ac-45d5-9242-aabb385cc5ad"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="f76aa77c-8923-4724-9a6d-d588cc513697"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>